<commit_message>
Correction taux accumulation après-retraite
</commit_message>
<xml_diff>
--- a/srpp/params/cpp_history.xlsx
+++ b/srpp/params/cpp_history.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\80002036\Documents\GitHub\srpp\srpp\params\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4603D996-D920-4F03-9977-E73E56E75C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EACE01DA-B95B-48C5-83E7-E25E741F2989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4826,7 +4826,7 @@
         <v>70</v>
       </c>
       <c r="O49" s="2">
-        <v>0.12891520244461421</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="P49" s="1">
         <v>0.75</v>
@@ -4915,7 +4915,7 @@
         <v>70</v>
       </c>
       <c r="O50" s="2">
-        <v>0.12842671614100179</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="P50" s="1">
         <v>0.75</v>
@@ -5004,7 +5004,7 @@
         <v>70</v>
       </c>
       <c r="O51" s="2">
-        <v>0.1288332426056977</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="P51" s="1">
         <v>0.75</v>
@@ -5093,7 +5093,7 @@
         <v>70</v>
       </c>
       <c r="O52" s="2">
-        <v>0.12881735644381559</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="P52" s="1">
         <v>0.75</v>
@@ -5182,7 +5182,7 @@
         <v>70</v>
       </c>
       <c r="O53" s="2">
-        <v>0.13035802035802041</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="P53" s="1">
         <v>0.75</v>
@@ -5271,7 +5271,7 @@
         <v>70</v>
       </c>
       <c r="O54" s="2">
-        <v>0.13117857969003011</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="P54" s="1">
         <v>0.75</v>
@@ -5360,6 +5360,9 @@
       <c r="N55" s="1">
         <v>70</v>
       </c>
+      <c r="O55" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P55" s="5">
         <v>0.75</v>
       </c>
@@ -5397,10 +5400,10 @@
         <v>0</v>
       </c>
       <c r="AB55" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC55" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
     <row r="56" spans="1:29" x14ac:dyDescent="0.25">
@@ -5447,6 +5450,9 @@
       <c r="N56" s="1">
         <v>70</v>
       </c>
+      <c r="O56" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P56" s="5">
         <v>0.75</v>
       </c>
@@ -5484,10 +5490,10 @@
         <v>0</v>
       </c>
       <c r="AB56" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC56" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
     <row r="57" spans="1:29" x14ac:dyDescent="0.25">
@@ -5534,6 +5540,9 @@
       <c r="N57" s="1">
         <v>70</v>
       </c>
+      <c r="O57" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P57" s="5">
         <v>0.75</v>
       </c>
@@ -5571,10 +5580,10 @@
         <v>0</v>
       </c>
       <c r="AB57" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC57" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
     <row r="58" spans="1:29" x14ac:dyDescent="0.25">
@@ -5620,6 +5629,9 @@
       <c r="N58" s="1">
         <v>70</v>
       </c>
+      <c r="O58" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P58" s="5">
         <v>0.75</v>
       </c>
@@ -5657,10 +5669,10 @@
         <v>0</v>
       </c>
       <c r="AB58" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC58" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
     <row r="59" spans="1:29" x14ac:dyDescent="0.25">
@@ -5706,6 +5718,9 @@
       <c r="N59" s="1">
         <v>70</v>
       </c>
+      <c r="O59" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P59" s="5">
         <v>0.75</v>
       </c>
@@ -5743,10 +5758,10 @@
         <v>0</v>
       </c>
       <c r="AB59" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC59" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
     <row r="60" spans="1:29" x14ac:dyDescent="0.25">
@@ -5792,6 +5807,9 @@
       <c r="N60" s="1">
         <v>70</v>
       </c>
+      <c r="O60" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P60" s="5">
         <v>0.75</v>
       </c>
@@ -5829,10 +5847,10 @@
         <v>0.33329999999999999</v>
       </c>
       <c r="AB60" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC60" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
     <row r="61" spans="1:29" x14ac:dyDescent="0.25">
@@ -5878,6 +5896,9 @@
       <c r="N61" s="1">
         <v>70</v>
       </c>
+      <c r="O61" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P61" s="5">
         <v>0.75</v>
       </c>
@@ -5915,10 +5936,10 @@
         <v>0.33329999999999999</v>
       </c>
       <c r="AB61" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC61" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
     <row r="62" spans="1:29" x14ac:dyDescent="0.25">
@@ -5964,6 +5985,9 @@
       <c r="N62" s="1">
         <v>70</v>
       </c>
+      <c r="O62" s="2">
+        <v>6.2500000000000003E-3</v>
+      </c>
       <c r="P62" s="5">
         <v>0.75</v>
       </c>
@@ -6001,10 +6025,10 @@
         <v>0.33329999999999999</v>
       </c>
       <c r="AB62" s="8">
-        <v>1.6000000000000001E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="AC62" s="8">
-        <v>6.6E-3</v>
+        <v>8.3300000000000006E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>